<commit_message>
alignment analysis and meme resultsç
</commit_message>
<xml_diff>
--- a/CollecTF_Output_Reports/80_Threshold_OUTPUT_REPORT/80_system_significance_matrix.xlsx
+++ b/CollecTF_Output_Reports/80_Threshold_OUTPUT_REPORT/80_system_significance_matrix.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J70"/>
+  <dimension ref="A1:L70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,6 +476,16 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>Sys_DR_Eval (Opt Thresh: 0.3729)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Sys_IR_Eval (Opt Thresh: 0.0052)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>Pipeline_Prediction</t>
         </is>
       </c>
@@ -520,6 +530,16 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
           <t>None (Insignificant)</t>
         </is>
       </c>
@@ -564,6 +584,16 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
           <t>None (Insignificant)</t>
         </is>
       </c>
@@ -608,6 +638,16 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
           <t>None (Insignificant)</t>
         </is>
       </c>
@@ -652,6 +692,16 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
           <t>IR</t>
         </is>
       </c>
@@ -696,6 +746,16 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
           <t>None (Insignificant)</t>
         </is>
       </c>
@@ -740,6 +800,16 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
           <t>IR</t>
         </is>
       </c>
@@ -784,6 +854,16 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
           <t>None (Insignificant)</t>
         </is>
       </c>
@@ -828,6 +908,16 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
           <t>DR</t>
         </is>
       </c>
@@ -872,6 +962,16 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
           <t>DR</t>
         </is>
       </c>
@@ -916,6 +1016,16 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
+          <t>FP</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>FN</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
           <t>DR</t>
         </is>
       </c>
@@ -960,6 +1070,16 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
           <t>None (Insignificant)</t>
         </is>
       </c>
@@ -1004,6 +1124,16 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
           <t>IR</t>
         </is>
       </c>
@@ -1048,6 +1178,16 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
           <t>IR</t>
         </is>
       </c>
@@ -1092,6 +1232,16 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
           <t>IR</t>
         </is>
       </c>
@@ -1136,6 +1286,16 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
           <t>IR</t>
         </is>
       </c>
@@ -1180,6 +1340,16 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
           <t>IR</t>
         </is>
       </c>
@@ -1224,6 +1394,16 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
           <t>None (Insignificant)</t>
         </is>
       </c>
@@ -1268,6 +1448,16 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
           <t>DR</t>
         </is>
       </c>
@@ -1312,6 +1502,16 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
           <t>IR</t>
         </is>
       </c>
@@ -1356,6 +1556,16 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
           <t>DR</t>
         </is>
       </c>
@@ -1400,6 +1610,16 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
           <t>DR</t>
         </is>
       </c>
@@ -1444,6 +1664,16 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
+          <t>FP</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>FN</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
           <t>None (Insignificant)</t>
         </is>
       </c>
@@ -1488,6 +1718,16 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
           <t>None (Insignificant)</t>
         </is>
       </c>
@@ -1532,6 +1772,16 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
           <t>IR</t>
         </is>
       </c>
@@ -1576,6 +1826,16 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
           <t>IR</t>
         </is>
       </c>
@@ -1620,6 +1880,16 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
           <t>None (Insignificant)</t>
         </is>
       </c>
@@ -1664,6 +1934,16 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
           <t>IR</t>
         </is>
       </c>
@@ -1708,6 +1988,16 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
           <t>IR</t>
         </is>
       </c>
@@ -1752,6 +2042,16 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
           <t>None (Insignificant)</t>
         </is>
       </c>
@@ -1796,6 +2096,16 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
           <t>IR</t>
         </is>
       </c>
@@ -1840,6 +2150,16 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
           <t>IR</t>
         </is>
       </c>
@@ -1884,6 +2204,16 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
           <t>IR</t>
         </is>
       </c>
@@ -1928,6 +2258,16 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
           <t>None (Insignificant)</t>
         </is>
       </c>
@@ -1972,6 +2312,16 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
           <t>IR</t>
         </is>
       </c>
@@ -2016,6 +2366,16 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
           <t>None (Insignificant)</t>
         </is>
       </c>
@@ -2060,6 +2420,16 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
+          <t>FP</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>FN</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
           <t>None (Insignificant)</t>
         </is>
       </c>
@@ -2104,6 +2474,16 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
           <t>DR</t>
         </is>
       </c>
@@ -2148,6 +2528,16 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
           <t>IR</t>
         </is>
       </c>
@@ -2192,6 +2582,16 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
           <t>DR</t>
         </is>
       </c>
@@ -2236,6 +2636,16 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
           <t>IR</t>
         </is>
       </c>
@@ -2280,6 +2690,16 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
           <t>IR</t>
         </is>
       </c>
@@ -2324,6 +2744,16 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
           <t>DR</t>
         </is>
       </c>
@@ -2368,6 +2798,16 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
           <t>IR</t>
         </is>
       </c>
@@ -2412,6 +2852,16 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
           <t>DR</t>
         </is>
       </c>
@@ -2456,6 +2906,16 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
           <t>DR</t>
         </is>
       </c>
@@ -2500,6 +2960,16 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
           <t>DR</t>
         </is>
       </c>
@@ -2544,6 +3014,16 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
+          <t>FN</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
           <t>No candidates found</t>
         </is>
       </c>
@@ -2588,6 +3068,16 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
           <t>DR</t>
         </is>
       </c>
@@ -2632,6 +3122,16 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
           <t>DR</t>
         </is>
       </c>
@@ -2676,6 +3176,16 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
           <t>None (Insignificant)</t>
         </is>
       </c>
@@ -2720,6 +3230,16 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
           <t>DR</t>
         </is>
       </c>
@@ -2764,6 +3284,16 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
           <t>DR</t>
         </is>
       </c>
@@ -2808,6 +3338,16 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
           <t>IR</t>
         </is>
       </c>
@@ -2852,6 +3392,16 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
           <t>IR</t>
         </is>
       </c>
@@ -2896,6 +3446,16 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
           <t>IR</t>
         </is>
       </c>
@@ -2940,6 +3500,16 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
           <t>IR</t>
         </is>
       </c>
@@ -2984,6 +3554,16 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
           <t>None (Insignificant)</t>
         </is>
       </c>
@@ -3028,6 +3608,16 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
+          <t>FP</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>FN</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
           <t>None (Insignificant)</t>
         </is>
       </c>
@@ -3072,6 +3662,16 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
+          <t>FP</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>FN</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
           <t>None (Insignificant)</t>
         </is>
       </c>
@@ -3116,6 +3716,16 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
+          <t>FP</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>FN</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
           <t>DR</t>
         </is>
       </c>
@@ -3160,6 +3770,16 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
           <t>IR</t>
         </is>
       </c>
@@ -3204,6 +3824,16 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
           <t>IR</t>
         </is>
       </c>
@@ -3248,6 +3878,16 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
           <t>IR</t>
         </is>
       </c>
@@ -3292,6 +3932,16 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
           <t>DR</t>
         </is>
       </c>
@@ -3336,6 +3986,16 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
           <t>IR</t>
         </is>
       </c>
@@ -3380,6 +4040,16 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
           <t>DR</t>
         </is>
       </c>
@@ -3424,6 +4094,16 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
           <t>None (Insignificant)</t>
         </is>
       </c>
@@ -3468,6 +4148,16 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
+          <t>FN</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>FP</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
           <t>IR</t>
         </is>
       </c>
@@ -3511,6 +4201,16 @@
         </is>
       </c>
       <c r="J70" t="inlineStr">
+        <is>
+          <t>FN</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>FP</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
         <is>
           <t>None (Insignificant)</t>
         </is>

</xml_diff>